<commit_message>
write bugs in admin ,profile pages
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Bug Report.xlsx
+++ b/TestCases_Docs/Bug Report.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Videos\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CEF578-F64A-4754-B75C-BF1792F68CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Report" sheetId="4" r:id="rId1"/>
@@ -21,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="414">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1530,11 +1524,262 @@
   <si>
     <t>Cart quantity isn't reduced to available stock automatically  when Stock decreases before checkout</t>
   </si>
+  <si>
+    <t>Defect_Admin_001</t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> product name: jacket
+ photo: dress.jpg
+ description: olive green jacket
+ price:50 :
+ stock avaliability:2 
+ supplier id: 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.click on actions
+2.click add product
+3.Enter valid product data
+4.Click Save
+</t>
+  </si>
+  <si>
+    <t>jana</t>
+  </si>
+  <si>
+    <t>product list is displayed with product name,decription,  image ,price quantity,supplier id for each product</t>
+  </si>
+  <si>
+    <t>supplier id dosent appear</t>
+  </si>
+  <si>
+    <t>TC-Admin-012</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the product data in the admin's product page dosent contain supplier id </t>
+  </si>
+  <si>
+    <t>Defect_Admin_002</t>
+  </si>
+  <si>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>TC-Admin-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin can't add product with all valid data </t>
+  </si>
+  <si>
+    <t>1.click on actions
+2.click add product
+3.Enter valid product data
+4.Click Save</t>
+  </si>
+  <si>
+    <t>Product is added successfully and redirect admin 
+ to dashboard</t>
+  </si>
+  <si>
+    <t>pop up appear with "please enter valid data"</t>
+  </si>
+  <si>
+    <t>product didn't deleted and pop up message appear 
+"are you sure? "</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product is deleted </t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-002</t>
+  </si>
+  <si>
+    <t>TC-Admin-003</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>admin can't removeproduct without validation</t>
+  </si>
+  <si>
+    <t>Defect_Admin_003</t>
+  </si>
+  <si>
+    <t>1.click product 
+2.Select product
+3.Click Remove
+4.Confirm deletion</t>
+  </si>
+  <si>
+    <t>Existing product</t>
+  </si>
+  <si>
+    <t>Defect_Admin_004</t>
+  </si>
+  <si>
+    <t>customer did't added but different pop up message appear
+"error creating user"</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and customer account is not created</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-003</t>
+  </si>
+  <si>
+    <t>No duplicate customer account is created</t>
+  </si>
+  <si>
+    <t>Product is created</t>
+  </si>
+  <si>
+    <t>Product is deleted</t>
+  </si>
+  <si>
+    <t>1.click on actions section
+ 2.Click Add user
+3.Enter valid Username, existing Email, valid Password, and 4.click on customer radio button
+5.Click Save</t>
+  </si>
+  <si>
+    <t>Existing customer email</t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in and a customer account with the same email already exists</t>
+  </si>
+  <si>
+    <t>TC-Admin-006</t>
+  </si>
+  <si>
+    <t>Supplier did't added but different pop up message appear
+"error creating user"</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and supplier account is not created</t>
+  </si>
+  <si>
+    <t>No duplicate supplier account is created</t>
+  </si>
+  <si>
+    <t>1.click on actions section
+ 2.Click Add user
+3.Enter valid Username, existing Email, valid Password, and 4.click on supplier radio button
+5.Click Save</t>
+  </si>
+  <si>
+    <t>Existing supplier email</t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in and a supplier account with the same email already exists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">when we add duplicate supplier email unexpected message appear </t>
+  </si>
+  <si>
+    <t xml:space="preserve">when we add duplicate customer email unexpected message appear </t>
+  </si>
+  <si>
+    <t>Defect_Admin_005</t>
+  </si>
+  <si>
+    <t>TC-Admin-009</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-004</t>
+  </si>
+  <si>
+    <t>all points appear with these extra points:
+total price and reciever</t>
+  </si>
+  <si>
+    <t>Order list is displayed with Order ID, Customer Name, and Supplier Name for each order</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-006</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>Lists remain available for review</t>
+  </si>
+  <si>
+    <t>1.Navigate to dashbord
+2.click orders
+3.validate that all requirments of the order displayed</t>
+  </si>
+  <si>
+    <t>admin see in the order page extra details like total and customer email</t>
+  </si>
+  <si>
+    <t>Defect_Admin_006</t>
+  </si>
+  <si>
+    <t>TC-Admin-013</t>
+  </si>
+  <si>
+    <t>no message 
+appear</t>
+  </si>
+  <si>
+    <t>No product found message is displayed</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-008</t>
+  </si>
+  <si>
+    <t>1.click on search bar
+ 2.Enter a non-existing product name in
+3.Click Search button</t>
+  </si>
+  <si>
+    <t>No matching product is displayed</t>
+  </si>
+  <si>
+    <t>Non-existing product name</t>
+  </si>
+  <si>
+    <t>Existing order details</t>
+  </si>
+  <si>
+    <t>when admin search with unavalibale product no message appear</t>
+  </si>
+  <si>
+    <t>Defect_Admin_007</t>
+  </si>
+  <si>
+    <t>TC-Admin-020</t>
+  </si>
+  <si>
+    <t>wireframe</t>
+  </si>
+  <si>
+    <t>there is navbar and footer in pages</t>
+  </si>
+  <si>
+    <t>no navbar and footer in pages</t>
+  </si>
+  <si>
+    <t>1-login with admin account
+2-go to actions (add user page or add products page )or profile page</t>
+  </si>
+  <si>
+    <t>when admin go to add user page , add product page or profile there is navbar and footer in the page</t>
+  </si>
+  <si>
+    <t>Defect_Admin_008</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -1818,7 +2063,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2042,12 +2287,330 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{9EE1B2E8-56F1-4388-8F05-1A16A6AD4072}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="49">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2310,7 +2873,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530EE577-BC47-4F64-BBFD-E7A5116B0BEB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -2940,24 +3503,54 @@
       <c r="AE10" s="58"/>
     </row>
     <row r="11" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="61"/>
+      <c r="A11" s="41" t="s">
+        <v>341</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>350</v>
+      </c>
+      <c r="C11" s="61" t="s">
+        <v>342</v>
+      </c>
       <c r="D11" s="3"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="63"/>
+      <c r="E11" s="38" t="s">
+        <v>344</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="78" t="s">
+        <v>16</v>
+      </c>
       <c r="H11" s="68"/>
-      <c r="I11" s="65"/>
-      <c r="J11" s="52"/>
+      <c r="I11" s="65" t="s">
+        <v>346</v>
+      </c>
+      <c r="J11" s="52" t="s">
+        <v>347</v>
+      </c>
       <c r="K11" s="56"/>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
-      <c r="N11" s="56"/>
-      <c r="O11" s="46"/>
-      <c r="P11" s="70"/>
-      <c r="Q11" s="72"/>
-      <c r="R11" s="71"/>
+      <c r="L11" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="M11" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="N11" s="46" t="s">
+        <v>348</v>
+      </c>
+      <c r="O11" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="P11" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R11" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S11" s="57"/>
       <c r="T11" s="58"/>
       <c r="U11" s="58"/>
@@ -2973,24 +3566,58 @@
       <c r="AE11" s="58"/>
     </row>
     <row r="12" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="68"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="52"/>
+      <c r="A12" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="C12" s="61" t="s">
+        <v>342</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="81" t="s">
+        <v>372</v>
+      </c>
+      <c r="I12" s="64" t="s">
+        <v>356</v>
+      </c>
+      <c r="J12" s="52" t="s">
+        <v>357</v>
+      </c>
       <c r="K12" s="56"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
-      <c r="N12" s="56"/>
-      <c r="O12" s="46"/>
-      <c r="P12" s="70"/>
-      <c r="Q12" s="72"/>
-      <c r="R12" s="71"/>
+      <c r="L12" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="M12" s="46" t="s">
+        <v>352</v>
+      </c>
+      <c r="N12" s="46" t="s">
+        <v>353</v>
+      </c>
+      <c r="O12" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="P12" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q12" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R12" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S12" s="57"/>
       <c r="T12" s="58"/>
       <c r="U12" s="58"/>
@@ -3006,24 +3633,58 @@
       <c r="AE12" s="58"/>
     </row>
     <row r="13" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="69"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="52"/>
+      <c r="A13" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C13" s="61" t="s">
+        <v>342</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="82" t="s">
+        <v>373</v>
+      </c>
+      <c r="I13" s="64" t="s">
+        <v>359</v>
+      </c>
+      <c r="J13" s="52" t="s">
+        <v>358</v>
+      </c>
       <c r="K13" s="56"/>
-      <c r="L13" s="56"/>
-      <c r="M13" s="56"/>
-      <c r="N13" s="56"/>
-      <c r="O13" s="46"/>
-      <c r="P13" s="70"/>
-      <c r="Q13" s="72"/>
-      <c r="R13" s="71"/>
+      <c r="L13" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="M13" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="N13" s="46" t="s">
+        <v>361</v>
+      </c>
+      <c r="O13" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="P13" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q13" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R13" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S13" s="57"/>
       <c r="T13" s="58"/>
       <c r="U13" s="58"/>
@@ -3039,24 +3700,58 @@
       <c r="AE13" s="58"/>
     </row>
     <row r="14" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="63"/>
-      <c r="H14" s="69"/>
-      <c r="I14" s="64"/>
-      <c r="J14" s="52"/>
+      <c r="A14" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C14" s="61" t="s">
+        <v>376</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="82" t="s">
+        <v>371</v>
+      </c>
+      <c r="I14" s="64" t="s">
+        <v>369</v>
+      </c>
+      <c r="J14" s="52" t="s">
+        <v>368</v>
+      </c>
       <c r="K14" s="56"/>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="56"/>
-      <c r="O14" s="46"/>
-      <c r="P14" s="70"/>
-      <c r="Q14" s="72"/>
-      <c r="R14" s="71"/>
+      <c r="L14" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="M14" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="N14" s="46" t="s">
+        <v>377</v>
+      </c>
+      <c r="O14" s="46" t="s">
+        <v>370</v>
+      </c>
+      <c r="P14" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q14" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R14" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S14" s="57"/>
       <c r="T14" s="58"/>
       <c r="U14" s="58"/>
@@ -3072,24 +3767,58 @@
       <c r="AE14" s="58"/>
     </row>
     <row r="15" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="61"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="64"/>
-      <c r="J15" s="52"/>
+      <c r="A15" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C15" s="61" t="s">
+        <v>383</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="82" t="s">
+        <v>380</v>
+      </c>
+      <c r="I15" s="64" t="s">
+        <v>379</v>
+      </c>
+      <c r="J15" s="52" t="s">
+        <v>378</v>
+      </c>
       <c r="K15" s="56"/>
-      <c r="L15" s="56"/>
-      <c r="M15" s="56"/>
-      <c r="N15" s="56"/>
-      <c r="O15" s="46"/>
-      <c r="P15" s="70"/>
-      <c r="Q15" s="72"/>
-      <c r="R15" s="71"/>
+      <c r="L15" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="M15" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="N15" s="46" t="s">
+        <v>387</v>
+      </c>
+      <c r="O15" s="46" t="s">
+        <v>388</v>
+      </c>
+      <c r="P15" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q15" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R15" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S15" s="57"/>
       <c r="T15" s="58"/>
       <c r="U15" s="58"/>
@@ -3105,24 +3834,58 @@
       <c r="AE15" s="58"/>
     </row>
     <row r="16" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="63"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="64"/>
-      <c r="J16" s="52"/>
+      <c r="A16" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C16" s="61" t="s">
+        <v>342</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="81" t="s">
+        <v>393</v>
+      </c>
+      <c r="I16" s="64" t="s">
+        <v>390</v>
+      </c>
+      <c r="J16" s="52" t="s">
+        <v>389</v>
+      </c>
       <c r="K16" s="56"/>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="56"/>
-      <c r="O16" s="46"/>
-      <c r="P16" s="70"/>
-      <c r="Q16" s="72"/>
-      <c r="R16" s="71"/>
+      <c r="L16" s="46" t="s">
+        <v>392</v>
+      </c>
+      <c r="M16" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="N16" s="46" t="s">
+        <v>397</v>
+      </c>
+      <c r="O16" s="46" t="s">
+        <v>391</v>
+      </c>
+      <c r="P16" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q16" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R16" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S16" s="57"/>
       <c r="T16" s="58"/>
       <c r="U16" s="58"/>
@@ -3138,24 +3901,58 @@
       <c r="AE16" s="58"/>
     </row>
     <row r="17" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="64"/>
-      <c r="J17" s="52"/>
+      <c r="A17" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="C17" s="61" t="s">
+        <v>342</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="81" t="s">
+        <v>402</v>
+      </c>
+      <c r="I17" s="64" t="s">
+        <v>399</v>
+      </c>
+      <c r="J17" s="52" t="s">
+        <v>398</v>
+      </c>
       <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="56"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="70"/>
-      <c r="Q17" s="72"/>
-      <c r="R17" s="71"/>
+      <c r="L17" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="M17" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="N17" s="46" t="s">
+        <v>407</v>
+      </c>
+      <c r="O17" s="46" t="s">
+        <v>400</v>
+      </c>
+      <c r="P17" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q17" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R17" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S17" s="57"/>
       <c r="T17" s="58"/>
       <c r="U17" s="58"/>
@@ -3171,24 +3968,52 @@
       <c r="AE17" s="58"/>
     </row>
     <row r="18" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="61"/>
+      <c r="A18" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="C18" s="61" t="s">
+        <v>342</v>
+      </c>
       <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="63"/>
+      <c r="E18" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="63" t="s">
+        <v>16</v>
+      </c>
       <c r="H18" s="68"/>
-      <c r="I18" s="64"/>
-      <c r="J18" s="52"/>
+      <c r="I18" s="64" t="s">
+        <v>410</v>
+      </c>
+      <c r="J18" s="52" t="s">
+        <v>409</v>
+      </c>
       <c r="K18" s="56"/>
-      <c r="L18" s="56"/>
-      <c r="M18" s="56"/>
+      <c r="L18" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="M18" s="46" t="s">
+        <v>362</v>
+      </c>
       <c r="N18" s="56"/>
-      <c r="O18" s="46"/>
-      <c r="P18" s="70"/>
-      <c r="Q18" s="72"/>
-      <c r="R18" s="71"/>
+      <c r="O18" s="46" t="s">
+        <v>408</v>
+      </c>
+      <c r="P18" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q18" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R18" s="71" t="s">
+        <v>345</v>
+      </c>
       <c r="S18" s="57"/>
       <c r="T18" s="58"/>
       <c r="U18" s="58"/>
@@ -9601,34 +10426,80 @@
     </row>
   </sheetData>
   <phoneticPr fontId="22" type="noConversion"/>
-  <conditionalFormatting sqref="Q2:Q22">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="New">
+  <conditionalFormatting sqref="Q19:Q22 Q2:Q11">
+    <cfRule type="containsText" dxfId="48" priority="15" operator="containsText" text="New">
       <formula>NOT(ISERROR(SEARCH("New",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="New">
+    <cfRule type="containsText" dxfId="47" priority="16" operator="containsText" text="New">
       <formula>NOT(ISERROR(SEARCH("New",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="46" priority="17" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Fix">
+    <cfRule type="containsText" dxfId="45" priority="18" operator="containsText" text="Fix">
       <formula>NOT(ISERROR(SEARCH("Fix",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="Reopen">
+    <cfRule type="containsText" dxfId="44" priority="19" operator="containsText" text="Reopen">
       <formula>NOT(ISERROR(SEARCH("Reopen",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="43" priority="20" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="Reopen">
+    <cfRule type="containsText" dxfId="42" priority="21" operator="containsText" text="Reopen">
       <formula>NOT(ISERROR(SEARCH("Reopen",Q2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q12">
+    <cfRule type="containsText" dxfId="41" priority="8" operator="containsText" text="New">
+      <formula>NOT(ISERROR(SEARCH("New",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="40" priority="9" operator="containsText" text="New">
+      <formula>NOT(ISERROR(SEARCH("New",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="39" priority="10" operator="containsText" text="Closed">
+      <formula>NOT(ISERROR(SEARCH("Closed",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="38" priority="11" operator="containsText" text="Fix">
+      <formula>NOT(ISERROR(SEARCH("Fix",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="37" priority="12" operator="containsText" text="Reopen">
+      <formula>NOT(ISERROR(SEARCH("Reopen",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="36" priority="13" operator="containsText" text="Open">
+      <formula>NOT(ISERROR(SEARCH("Open",Q12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="35" priority="14" operator="containsText" text="Reopen">
+      <formula>NOT(ISERROR(SEARCH("Reopen",Q12)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q13:Q18">
+    <cfRule type="containsText" dxfId="34" priority="1" operator="containsText" text="New">
+      <formula>NOT(ISERROR(SEARCH("New",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="33" priority="2" operator="containsText" text="New">
+      <formula>NOT(ISERROR(SEARCH("New",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="32" priority="3" operator="containsText" text="Closed">
+      <formula>NOT(ISERROR(SEARCH("Closed",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="31" priority="4" operator="containsText" text="Fix">
+      <formula>NOT(ISERROR(SEARCH("Fix",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="30" priority="5" operator="containsText" text="Reopen">
+      <formula>NOT(ISERROR(SEARCH("Reopen",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="Open">
+      <formula>NOT(ISERROR(SEARCH("Open",Q13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="28" priority="7" operator="containsText" text="Reopen">
+      <formula>NOT(ISERROR(SEARCH("Reopen",Q13)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F22" xr:uid="{872A2AB6-2ADB-4D3A-9A56-79D755130126}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F22">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q22" xr:uid="{7A9CF52A-021F-4101-8226-913AE7D0D2C0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q22">
       <formula1>"New, Open, Fix, Reopen, Closed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9638,7 +10509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -15162,20 +16033,20 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q2:Q979" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q2:Q979">
       <formula1>"not executed,blocked,failed,passed"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
-    <hyperlink ref="E9" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
-    <hyperlink ref="E36" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
+    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="E7" r:id="rId6"/>
+    <hyperlink ref="E8" r:id="rId7"/>
+    <hyperlink ref="E9" r:id="rId8"/>
+    <hyperlink ref="E36" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
test/update bug report add checkout bugs
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Bug Report.xlsx
+++ b/TestCases_Docs/Bug Report.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A439B612-3ECE-42A9-9B6B-2515A1DD1CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
+    <workbookView xWindow="0" yWindow="900" windowWidth="23040" windowHeight="7044" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Report" sheetId="4" r:id="rId1"/>
@@ -15,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="443">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1525,10 +1531,141 @@
     <t>Cart quantity isn't reduced to available stock automatically  when Stock decreases before checkout</t>
   </si>
   <si>
+    <t>Defect_CHK_001</t>
+  </si>
+  <si>
+    <t>Defect_CHK_002</t>
+  </si>
+  <si>
+    <t>Defect_CHK_003</t>
+  </si>
+  <si>
+    <t>Defect_CHK_004</t>
+  </si>
+  <si>
+    <t>Defect_CHK_005</t>
+  </si>
+  <si>
+    <t>Verify City field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>Verify Address field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t>Verify successful checkout with valid data
+(city, Address, Mobile phone of reciever, name's reciever, Email)</t>
+  </si>
+  <si>
+    <t>SRS-FN- Checkout-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRS-FN-Checkout-002
+</t>
+  </si>
+  <si>
+    <t>SRS-FN-Checkout-002</t>
+  </si>
+  <si>
+    <t>open URL
+User logged in</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Leave City field empty
+6. Enter Address 
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City
+6. Leave Address field empty
+7. Enter phone of reciever
+8.Enter name of reciever
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field 
+6. Enter Address field
+7. Enter phone of reciever
+8.leave name of reciever empty
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field
+6. Enter Address field
+7. Leave phone of reciever
+8.Enter name of reciever 
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>1. Select product from home page 
+2. Add product to cart
+3. Open cart 
+4. Click checkout
+5. Enter City field 
+6. Enter Address field 
+7. Enter phone of reciever
+8.Enter name of reciever 
+9. Click confirm Order button</t>
+  </si>
+  <si>
+    <t>Verify name of reciever name field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify phone of reciever phone field is mandatory when left empty with other valid data</t>
+  </si>
+  <si>
     <t>Defect_Admin_001</t>
   </si>
   <si>
+    <t xml:space="preserve">the product data in the admin's product page dosent contain supplier id </t>
+  </si>
+  <si>
     <t>Open URL, Admin is logged in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.click on actions
+2.click add product
+3.Enter valid product data
+4.Click Save
+</t>
+  </si>
+  <si>
+    <t>product list is displayed with product name,decription,  image ,price quantity,supplier id for each product</t>
+  </si>
+  <si>
+    <t>supplier id dosent appear</t>
+  </si>
+  <si>
+    <t>TC-Admin-012</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-001</t>
+  </si>
+  <si>
+    <t>jana</t>
+  </si>
+  <si>
+    <t>Defect_Admin_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin can't add product with all valid data </t>
   </si>
   <si>
     <t xml:space="preserve"> product name: jacket
@@ -1539,49 +1676,15 @@
  supplier id: 16</t>
   </si>
   <si>
-    <t xml:space="preserve">1.click on actions
-2.click add product
-3.Enter valid product data
-4.Click Save
-</t>
-  </si>
-  <si>
-    <t>jana</t>
-  </si>
-  <si>
-    <t>product list is displayed with product name,decription,  image ,price quantity,supplier id for each product</t>
-  </si>
-  <si>
-    <t>supplier id dosent appear</t>
-  </si>
-  <si>
-    <t>TC-Admin-012</t>
-  </si>
-  <si>
-    <t>SRS-FN-Admin-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the product data in the admin's product page dosent contain supplier id </t>
-  </si>
-  <si>
-    <t>Defect_Admin_002</t>
-  </si>
-  <si>
-    <t>critical</t>
-  </si>
-  <si>
-    <t>TC-Admin-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">admin can't add product with all valid data </t>
-  </si>
-  <si>
     <t>1.click on actions
 2.click add product
 3.Enter valid product data
 4.Click Save</t>
   </si>
   <si>
+    <t>Product is created</t>
+  </si>
+  <si>
     <t>Product is added successfully and redirect admin 
  to dashboard</t>
   </si>
@@ -1589,26 +1692,19 @@
     <t>pop up appear with "please enter valid data"</t>
   </si>
   <si>
-    <t>product didn't deleted and pop up message appear 
-"are you sure? "</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product is deleted </t>
-  </si>
-  <si>
-    <t>SRS-FN-Admin-002</t>
-  </si>
-  <si>
-    <t>TC-Admin-003</t>
-  </si>
-  <si>
-    <t>low</t>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>TC-Admin-01</t>
+  </si>
+  <si>
+    <t>Defect_Admin_003</t>
   </si>
   <si>
     <t>admin can't removeproduct without validation</t>
   </si>
   <si>
-    <t>Defect_Admin_003</t>
+    <t>Existing product</t>
   </si>
   <si>
     <t>1.click product 
@@ -1617,29 +1713,35 @@
 4.Confirm deletion</t>
   </si>
   <si>
-    <t>Existing product</t>
+    <t>Product is deleted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product is deleted </t>
+  </si>
+  <si>
+    <t>product didn't deleted and pop up message appear 
+"are you sure? "</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>TC-Admin-003</t>
+  </si>
+  <si>
+    <t>SRS-FN-Admin-002</t>
   </si>
   <si>
     <t>Defect_Admin_004</t>
   </si>
   <si>
-    <t>customer did't added but different pop up message appear
-"error creating user"</t>
-  </si>
-  <si>
-    <t>System shows "Email already exists" message and customer account is not created</t>
-  </si>
-  <si>
-    <t>SRS-FN-Admin-003</t>
-  </si>
-  <si>
-    <t>No duplicate customer account is created</t>
-  </si>
-  <si>
-    <t>Product is created</t>
-  </si>
-  <si>
-    <t>Product is deleted</t>
+    <t xml:space="preserve">when we add duplicate customer email unexpected message appear </t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in and a customer account with the same email already exists</t>
+  </si>
+  <si>
+    <t>Existing customer email</t>
   </si>
   <si>
     <t>1.click on actions section
@@ -1648,23 +1750,32 @@
 5.Click Save</t>
   </si>
   <si>
-    <t>Existing customer email</t>
-  </si>
-  <si>
-    <t>Open URL, Admin is logged in and a customer account with the same email already exists</t>
+    <t>No duplicate customer account is created</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and customer account is not created</t>
+  </si>
+  <si>
+    <t>customer did't added but different pop up message appear
+"error creating user"</t>
   </si>
   <si>
     <t>TC-Admin-006</t>
   </si>
   <si>
-    <t>Supplier did't added but different pop up message appear
-"error creating user"</t>
-  </si>
-  <si>
-    <t>System shows "Email already exists" message and supplier account is not created</t>
-  </si>
-  <si>
-    <t>No duplicate supplier account is created</t>
+    <t>SRS-FN-Admin-003</t>
+  </si>
+  <si>
+    <t>Defect_Admin_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">when we add duplicate supplier email unexpected message appear </t>
+  </si>
+  <si>
+    <t>Open URL, Admin is logged in and a supplier account with the same email already exists</t>
+  </si>
+  <si>
+    <t>Existing supplier email</t>
   </si>
   <si>
     <t>1.click on actions section
@@ -1673,19 +1784,14 @@
 5.Click Save</t>
   </si>
   <si>
-    <t>Existing supplier email</t>
-  </si>
-  <si>
-    <t>Open URL, Admin is logged in and a supplier account with the same email already exists</t>
-  </si>
-  <si>
-    <t xml:space="preserve">when we add duplicate supplier email unexpected message appear </t>
-  </si>
-  <si>
-    <t xml:space="preserve">when we add duplicate customer email unexpected message appear </t>
-  </si>
-  <si>
-    <t>Defect_Admin_005</t>
+    <t>No duplicate supplier account is created</t>
+  </si>
+  <si>
+    <t>System shows "Email already exists" message and supplier account is not created</t>
+  </si>
+  <si>
+    <t>Supplier did't added but different pop up message appear
+"error creating user"</t>
   </si>
   <si>
     <t>TC-Admin-009</t>
@@ -1694,20 +1800,13 @@
     <t>SRS-FN-Admin-004</t>
   </si>
   <si>
-    <t>all points appear with these extra points:
-total price and reciever</t>
-  </si>
-  <si>
-    <t>Order list is displayed with Order ID, Customer Name, and Supplier Name for each order</t>
-  </si>
-  <si>
-    <t>SRS-FN-Admin-006</t>
-  </si>
-  <si>
-    <t>medium</t>
-  </si>
-  <si>
-    <t>Lists remain available for review</t>
+    <t>Defect_Admin_006</t>
+  </si>
+  <si>
+    <t>admin see in the order page extra details like total and customer email</t>
+  </si>
+  <si>
+    <t>Existing order details</t>
   </si>
   <si>
     <t>1.Navigate to dashbord
@@ -1715,23 +1814,32 @@
 3.validate that all requirments of the order displayed</t>
   </si>
   <si>
-    <t>admin see in the order page extra details like total and customer email</t>
-  </si>
-  <si>
-    <t>Defect_Admin_006</t>
+    <t>Lists remain available for review</t>
+  </si>
+  <si>
+    <t>Order list is displayed with Order ID, Customer Name, and Supplier Name for each order</t>
+  </si>
+  <si>
+    <t>all points appear with these extra points:
+total price and reciever</t>
+  </si>
+  <si>
+    <t>medium</t>
   </si>
   <si>
     <t>TC-Admin-013</t>
   </si>
   <si>
-    <t>no message 
-appear</t>
-  </si>
-  <si>
-    <t>No product found message is displayed</t>
-  </si>
-  <si>
-    <t>SRS-FN-Admin-008</t>
+    <t>SRS-FN-Admin-006</t>
+  </si>
+  <si>
+    <t>Defect_Admin_007</t>
+  </si>
+  <si>
+    <t>when admin search with unavalibale product no message appear</t>
+  </si>
+  <si>
+    <t>Non-existing product name</t>
   </si>
   <si>
     <t>1.click on search bar
@@ -1742,45 +1850,80 @@
     <t>No matching product is displayed</t>
   </si>
   <si>
-    <t>Non-existing product name</t>
-  </si>
-  <si>
-    <t>Existing order details</t>
-  </si>
-  <si>
-    <t>when admin search with unavalibale product no message appear</t>
-  </si>
-  <si>
-    <t>Defect_Admin_007</t>
+    <t>No product found message is displayed</t>
+  </si>
+  <si>
+    <t>no message 
+appear</t>
   </si>
   <si>
     <t>TC-Admin-020</t>
   </si>
   <si>
-    <t>wireframe</t>
-  </si>
-  <si>
-    <t>there is navbar and footer in pages</t>
-  </si>
-  <si>
-    <t>no navbar and footer in pages</t>
+    <t>SRS-FN-Admin-008</t>
+  </si>
+  <si>
+    <t>Defect_Admin_008</t>
+  </si>
+  <si>
+    <t>when admin go to add user page , add product page or profile there is navbar and footer in the page</t>
   </si>
   <si>
     <t>1-login with admin account
 2-go to actions (add user page or add products page )or profile page</t>
   </si>
   <si>
-    <t>when admin go to add user page , add product page or profile there is navbar and footer in the page</t>
-  </si>
-  <si>
-    <t>Defect_Admin_008</t>
+    <t>no navbar and footer in pages</t>
+  </si>
+  <si>
+    <t>there is navbar and footer in pages</t>
+  </si>
+  <si>
+    <t>wireframe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user is redirected to home page and pop up message "Order is placed successfully" 
+</t>
+  </si>
+  <si>
+    <t>no popup message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pop up message appears
+"Please Enter the required data"
+ and order is not placed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no pop up message appears "Please Enter the required data"
+</t>
+  </si>
+  <si>
+    <t>pop up message appears
+"Please Enter the required data"
+ and order is not placed</t>
+  </si>
+  <si>
+    <t>TC_CHK_001</t>
+  </si>
+  <si>
+    <t>TC_CHK_003</t>
+  </si>
+  <si>
+    <t>TC_CHK_004</t>
+  </si>
+  <si>
+    <t>TC_CHK_005</t>
+  </si>
+  <si>
+    <t>TC_CHK_006</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="23" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1916,6 +2059,19 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -2059,11 +2215,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2287,330 +2456,79 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="15">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 10" xfId="9" xr:uid="{832D0BBE-823B-4EE1-8AD4-72D8A89C2F73}"/>
+    <cellStyle name="Normal 11" xfId="10" xr:uid="{3D5C94BC-A247-4B45-917B-A4274E0542D5}"/>
+    <cellStyle name="Normal 12" xfId="11" xr:uid="{3B0A0E51-A249-4CA5-A4DB-F62439F8BB8E}"/>
+    <cellStyle name="Normal 13" xfId="12" xr:uid="{F5408A00-0B76-4E73-8B1E-DDDE739CB25B}"/>
+    <cellStyle name="Normal 14" xfId="13" xr:uid="{57BBBDEB-0AD6-4988-A50D-708126049A8F}"/>
+    <cellStyle name="Normal 15" xfId="14" xr:uid="{6BE7F390-4FE6-4DA2-ABD6-ECE2CE9CD309}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{9EE1B2E8-56F1-4388-8F05-1A16A6AD4072}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{C26CAA55-5F0D-4A90-A11E-A8D20D679B09}"/>
+    <cellStyle name="Normal 4" xfId="3" xr:uid="{A27B9F2B-BBA3-4A08-AF7B-F6CFD0846F73}"/>
+    <cellStyle name="Normal 5" xfId="4" xr:uid="{2A6D86B2-0E2A-4EFB-A8F1-DEBC2095CCFD}"/>
+    <cellStyle name="Normal 6" xfId="5" xr:uid="{793DB909-FCEE-44ED-A466-8993481756E9}"/>
+    <cellStyle name="Normal 7" xfId="6" xr:uid="{D67A7D59-1B8B-437A-AB41-09DDC120947A}"/>
+    <cellStyle name="Normal 8" xfId="7" xr:uid="{459B37FB-7BCD-494F-A52B-7CCE1374E4B9}"/>
+    <cellStyle name="Normal 9" xfId="8" xr:uid="{4CE399EB-C99B-4AC2-AC21-3736EFC3EFB1}"/>
   </cellStyles>
-  <dxfs count="49">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
@@ -2873,11 +2791,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530EE577-BC47-4F64-BBFD-E7A5116B0BEB}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AE1000"/>
+  <dimension ref="A1:AE1007"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.109375" style="45" customWidth="1"/>
@@ -2886,7 +2804,7 @@
     <col min="4" max="4" width="32.6640625" style="45" customWidth="1"/>
     <col min="5" max="5" width="78.109375" style="45" customWidth="1"/>
     <col min="6" max="6" width="24" style="45" customWidth="1"/>
-    <col min="7" max="7" width="22" style="45" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" style="45" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="56.33203125" style="45" customWidth="1"/>
     <col min="9" max="9" width="78.109375" style="45" customWidth="1"/>
     <col min="10" max="10" width="76.6640625" style="45" customWidth="1"/>
@@ -2918,7 +2836,7 @@
       <c r="G1" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="43" t="s">
+      <c r="H1" s="95" t="s">
         <v>274</v>
       </c>
       <c r="I1" s="43" t="s">
@@ -3450,7 +3368,7 @@
       <c r="D10" s="76" t="s">
         <v>331</v>
       </c>
-      <c r="E10" s="40" t="s">
+      <c r="E10" s="85" t="s">
         <v>333</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -3504,17 +3422,17 @@
     </row>
     <row r="11" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>350</v>
+        <v>361</v>
       </c>
       <c r="C11" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="38" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>15</v>
@@ -3524,10 +3442,10 @@
       </c>
       <c r="H11" s="68"/>
       <c r="I11" s="65" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="J11" s="52" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="K11" s="56"/>
       <c r="L11" s="46" t="s">
@@ -3537,10 +3455,10 @@
         <v>291</v>
       </c>
       <c r="N11" s="46" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="O11" s="46" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="P11" s="70" t="s">
         <v>26</v>
@@ -3549,7 +3467,7 @@
         <v>281</v>
       </c>
       <c r="R11" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S11" s="57"/>
       <c r="T11" s="58"/>
@@ -3567,19 +3485,19 @@
     </row>
     <row r="12" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="C12" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>343</v>
+        <v>371</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>355</v>
+        <v>372</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>15</v>
@@ -3587,27 +3505,27 @@
       <c r="G12" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="81" t="s">
-        <v>372</v>
+      <c r="H12" s="93" t="s">
+        <v>373</v>
       </c>
       <c r="I12" s="64" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="J12" s="52" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="K12" s="56"/>
       <c r="L12" s="46" t="s">
         <v>300</v>
       </c>
       <c r="M12" s="46" t="s">
-        <v>352</v>
+        <v>376</v>
       </c>
       <c r="N12" s="46" t="s">
-        <v>353</v>
+        <v>377</v>
       </c>
       <c r="O12" s="46" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="P12" s="70" t="s">
         <v>26</v>
@@ -3616,7 +3534,7 @@
         <v>281</v>
       </c>
       <c r="R12" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S12" s="57"/>
       <c r="T12" s="58"/>
@@ -3634,19 +3552,19 @@
     </row>
     <row r="13" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
       <c r="C13" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>15</v>
@@ -3654,27 +3572,27 @@
       <c r="G13" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="82" t="s">
-        <v>373</v>
+      <c r="H13" s="94" t="s">
+        <v>382</v>
       </c>
       <c r="I13" s="64" t="s">
-        <v>359</v>
+        <v>383</v>
       </c>
       <c r="J13" s="52" t="s">
-        <v>358</v>
+        <v>384</v>
       </c>
       <c r="K13" s="56"/>
       <c r="L13" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="M13" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="N13" s="46" t="s">
-        <v>361</v>
+        <v>386</v>
       </c>
       <c r="O13" s="46" t="s">
-        <v>360</v>
+        <v>387</v>
       </c>
       <c r="P13" s="70" t="s">
         <v>26</v>
@@ -3683,7 +3601,7 @@
         <v>281</v>
       </c>
       <c r="R13" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S13" s="57"/>
       <c r="T13" s="58"/>
@@ -3701,19 +3619,19 @@
     </row>
     <row r="14" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>367</v>
+        <v>388</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C14" s="61" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>15</v>
@@ -3721,14 +3639,14 @@
       <c r="G14" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="82" t="s">
-        <v>371</v>
+      <c r="H14" s="94" t="s">
+        <v>393</v>
       </c>
       <c r="I14" s="64" t="s">
-        <v>369</v>
+        <v>394</v>
       </c>
       <c r="J14" s="52" t="s">
-        <v>368</v>
+        <v>395</v>
       </c>
       <c r="K14" s="56"/>
       <c r="L14" s="46" t="s">
@@ -3738,10 +3656,10 @@
         <v>300</v>
       </c>
       <c r="N14" s="46" t="s">
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="O14" s="46" t="s">
-        <v>370</v>
+        <v>397</v>
       </c>
       <c r="P14" s="70" t="s">
         <v>26</v>
@@ -3750,7 +3668,7 @@
         <v>281</v>
       </c>
       <c r="R14" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S14" s="57"/>
       <c r="T14" s="58"/>
@@ -3768,19 +3686,19 @@
     </row>
     <row r="15" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="C15" s="61" t="s">
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>381</v>
+        <v>402</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>15</v>
@@ -3788,14 +3706,14 @@
       <c r="G15" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="82" t="s">
-        <v>380</v>
+      <c r="H15" s="94" t="s">
+        <v>403</v>
       </c>
       <c r="I15" s="64" t="s">
-        <v>379</v>
+        <v>404</v>
       </c>
       <c r="J15" s="52" t="s">
-        <v>378</v>
+        <v>405</v>
       </c>
       <c r="K15" s="56"/>
       <c r="L15" s="46" t="s">
@@ -3805,10 +3723,10 @@
         <v>300</v>
       </c>
       <c r="N15" s="46" t="s">
-        <v>387</v>
+        <v>406</v>
       </c>
       <c r="O15" s="46" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
       <c r="P15" s="70" t="s">
         <v>26</v>
@@ -3817,7 +3735,7 @@
         <v>281</v>
       </c>
       <c r="R15" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S15" s="57"/>
       <c r="T15" s="58"/>
@@ -3835,19 +3753,19 @@
     </row>
     <row r="16" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>395</v>
+        <v>409</v>
       </c>
       <c r="C16" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>394</v>
+        <v>411</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>15</v>
@@ -3855,27 +3773,27 @@
       <c r="G16" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="81" t="s">
-        <v>393</v>
+      <c r="H16" s="93" t="s">
+        <v>412</v>
       </c>
       <c r="I16" s="64" t="s">
-        <v>390</v>
+        <v>413</v>
       </c>
       <c r="J16" s="52" t="s">
-        <v>389</v>
+        <v>414</v>
       </c>
       <c r="K16" s="56"/>
       <c r="L16" s="46" t="s">
-        <v>392</v>
+        <v>415</v>
       </c>
       <c r="M16" s="46" t="s">
         <v>291</v>
       </c>
       <c r="N16" s="46" t="s">
-        <v>397</v>
+        <v>416</v>
       </c>
       <c r="O16" s="46" t="s">
-        <v>391</v>
+        <v>417</v>
       </c>
       <c r="P16" s="70" t="s">
         <v>26</v>
@@ -3884,7 +3802,7 @@
         <v>281</v>
       </c>
       <c r="R16" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S16" s="57"/>
       <c r="T16" s="58"/>
@@ -3902,19 +3820,19 @@
     </row>
     <row r="17" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>405</v>
+        <v>419</v>
       </c>
       <c r="C17" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>401</v>
+        <v>421</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>15</v>
@@ -3922,27 +3840,27 @@
       <c r="G17" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="81" t="s">
-        <v>402</v>
+      <c r="H17" s="93" t="s">
+        <v>422</v>
       </c>
       <c r="I17" s="64" t="s">
-        <v>399</v>
+        <v>423</v>
       </c>
       <c r="J17" s="52" t="s">
-        <v>398</v>
+        <v>424</v>
       </c>
       <c r="K17" s="56"/>
       <c r="L17" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="M17" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="N17" s="46" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
       <c r="O17" s="46" t="s">
-        <v>400</v>
+        <v>426</v>
       </c>
       <c r="P17" s="70" t="s">
         <v>26</v>
@@ -3951,7 +3869,7 @@
         <v>281</v>
       </c>
       <c r="R17" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S17" s="57"/>
       <c r="T17" s="58"/>
@@ -3969,17 +3887,17 @@
     </row>
     <row r="18" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>413</v>
+        <v>427</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="C18" s="61" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>15</v>
@@ -3989,21 +3907,21 @@
       </c>
       <c r="H18" s="68"/>
       <c r="I18" s="64" t="s">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="J18" s="52" t="s">
-        <v>409</v>
+        <v>431</v>
       </c>
       <c r="K18" s="56"/>
       <c r="L18" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="M18" s="46" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="N18" s="56"/>
       <c r="O18" s="46" t="s">
-        <v>408</v>
+        <v>432</v>
       </c>
       <c r="P18" s="70" t="s">
         <v>26</v>
@@ -4012,7 +3930,7 @@
         <v>281</v>
       </c>
       <c r="R18" s="71" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="S18" s="57"/>
       <c r="T18" s="58"/>
@@ -4029,24 +3947,56 @@
       <c r="AE18" s="58"/>
     </row>
     <row r="19" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="69"/>
-      <c r="I19" s="65"/>
-      <c r="J19" s="52"/>
+      <c r="A19" s="41" t="s">
+        <v>341</v>
+      </c>
+      <c r="B19" s="84" t="s">
+        <v>348</v>
+      </c>
+      <c r="C19" s="89" t="s">
+        <v>352</v>
+      </c>
+      <c r="D19" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="E19" s="91" t="s">
+        <v>353</v>
+      </c>
+      <c r="F19" s="81" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="68"/>
+      <c r="I19" s="96" t="s">
+        <v>433</v>
+      </c>
+      <c r="J19" s="97" t="s">
+        <v>434</v>
+      </c>
       <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
-      <c r="M19" s="56"/>
-      <c r="N19" s="56"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="70"/>
-      <c r="Q19" s="72"/>
-      <c r="R19" s="71"/>
+      <c r="L19" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="M19" s="46" t="s">
+        <v>301</v>
+      </c>
+      <c r="N19" s="98" t="s">
+        <v>438</v>
+      </c>
+      <c r="O19" s="86" t="s">
+        <v>349</v>
+      </c>
+      <c r="P19" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q19" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R19" s="71" t="s">
+        <v>17</v>
+      </c>
       <c r="S19" s="57"/>
       <c r="T19" s="58"/>
       <c r="U19" s="58"/>
@@ -4062,24 +4012,56 @@
       <c r="AE19" s="58"/>
     </row>
     <row r="20" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="63"/>
-      <c r="H20" s="69"/>
-      <c r="I20" s="64"/>
-      <c r="J20" s="52"/>
+      <c r="A20" s="41" t="s">
+        <v>342</v>
+      </c>
+      <c r="B20" s="83" t="s">
+        <v>346</v>
+      </c>
+      <c r="C20" s="89" t="s">
+        <v>352</v>
+      </c>
+      <c r="D20" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="E20" s="91" t="s">
+        <v>354</v>
+      </c>
+      <c r="F20" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="68"/>
+      <c r="I20" s="96" t="s">
+        <v>435</v>
+      </c>
+      <c r="J20" s="96" t="s">
+        <v>436</v>
+      </c>
       <c r="K20" s="56"/>
-      <c r="L20" s="56"/>
-      <c r="M20" s="56"/>
-      <c r="N20" s="56"/>
-      <c r="O20" s="46"/>
-      <c r="P20" s="70"/>
-      <c r="Q20" s="72"/>
-      <c r="R20" s="71"/>
+      <c r="L20" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="M20" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="N20" s="98" t="s">
+        <v>439</v>
+      </c>
+      <c r="O20" s="88" t="s">
+        <v>350</v>
+      </c>
+      <c r="P20" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q20" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R20" s="71" t="s">
+        <v>17</v>
+      </c>
       <c r="S20" s="57"/>
       <c r="T20" s="58"/>
       <c r="U20" s="58"/>
@@ -4095,24 +4077,56 @@
       <c r="AE20" s="58"/>
     </row>
     <row r="21" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="63"/>
+      <c r="A21" s="41" t="s">
+        <v>343</v>
+      </c>
+      <c r="B21" s="83" t="s">
+        <v>347</v>
+      </c>
+      <c r="C21" s="89" t="s">
+        <v>352</v>
+      </c>
+      <c r="D21" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="E21" s="91" t="s">
+        <v>355</v>
+      </c>
+      <c r="F21" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="78" t="s">
+        <v>16</v>
+      </c>
       <c r="H21" s="69"/>
-      <c r="I21" s="64"/>
-      <c r="J21" s="52"/>
+      <c r="I21" s="96" t="s">
+        <v>437</v>
+      </c>
+      <c r="J21" s="96" t="s">
+        <v>436</v>
+      </c>
       <c r="K21" s="56"/>
-      <c r="L21" s="56"/>
-      <c r="M21" s="56"/>
-      <c r="N21" s="56"/>
-      <c r="O21" s="46"/>
-      <c r="P21" s="70"/>
-      <c r="Q21" s="72"/>
-      <c r="R21" s="71"/>
+      <c r="L21" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="M21" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="N21" s="98" t="s">
+        <v>440</v>
+      </c>
+      <c r="O21" s="87" t="s">
+        <v>351</v>
+      </c>
+      <c r="P21" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q21" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R21" s="71" t="s">
+        <v>17</v>
+      </c>
       <c r="S21" s="57"/>
       <c r="T21" s="58"/>
       <c r="U21" s="58"/>
@@ -4128,24 +4142,56 @@
       <c r="AE21" s="58"/>
     </row>
     <row r="22" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="61"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="63"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="64"/>
-      <c r="J22" s="52"/>
+      <c r="A22" s="41" t="s">
+        <v>344</v>
+      </c>
+      <c r="B22" s="83" t="s">
+        <v>358</v>
+      </c>
+      <c r="C22" s="89" t="s">
+        <v>352</v>
+      </c>
+      <c r="D22" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="E22" s="91" t="s">
+        <v>356</v>
+      </c>
+      <c r="F22" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="69"/>
+      <c r="I22" s="96" t="s">
+        <v>437</v>
+      </c>
+      <c r="J22" s="96" t="s">
+        <v>436</v>
+      </c>
       <c r="K22" s="56"/>
-      <c r="L22" s="56"/>
-      <c r="M22" s="56"/>
-      <c r="N22" s="56"/>
-      <c r="O22" s="46"/>
-      <c r="P22" s="70"/>
-      <c r="Q22" s="72"/>
-      <c r="R22" s="71"/>
+      <c r="L22" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="M22" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="N22" s="98" t="s">
+        <v>441</v>
+      </c>
+      <c r="O22" s="87" t="s">
+        <v>351</v>
+      </c>
+      <c r="P22" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q22" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R22" s="71" t="s">
+        <v>17</v>
+      </c>
       <c r="S22" s="57"/>
       <c r="T22" s="58"/>
       <c r="U22" s="58"/>
@@ -4160,61 +4206,268 @@
       <c r="AD22" s="58"/>
       <c r="AE22" s="58"/>
     </row>
-    <row r="23" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E23" s="59"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="60"/>
-      <c r="O23" s="60"/>
-      <c r="R23" s="60"/>
-      <c r="S23" s="59"/>
-    </row>
-    <row r="24" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E24" s="59"/>
-      <c r="I24" s="59"/>
-      <c r="J24" s="60"/>
-      <c r="O24" s="60"/>
-      <c r="R24" s="60"/>
-      <c r="S24" s="59"/>
-    </row>
-    <row r="25" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E25" s="59"/>
-      <c r="I25" s="59"/>
-      <c r="J25" s="60"/>
-      <c r="O25" s="60"/>
-      <c r="R25" s="60"/>
-      <c r="S25" s="59"/>
-    </row>
-    <row r="26" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="60"/>
-      <c r="O26" s="60"/>
-      <c r="R26" s="60"/>
-      <c r="S26" s="59"/>
-    </row>
-    <row r="27" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E27" s="59"/>
-      <c r="I27" s="59"/>
-      <c r="J27" s="60"/>
-      <c r="O27" s="60"/>
-      <c r="R27" s="60"/>
-      <c r="S27" s="59"/>
-    </row>
-    <row r="28" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E28" s="59"/>
-      <c r="I28" s="59"/>
-      <c r="J28" s="60"/>
-      <c r="O28" s="60"/>
-      <c r="R28" s="60"/>
-      <c r="S28" s="59"/>
-    </row>
-    <row r="29" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E29" s="59"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="60"/>
-      <c r="O29" s="60"/>
-      <c r="R29" s="60"/>
-      <c r="S29" s="59"/>
+    <row r="23" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="41" t="s">
+        <v>345</v>
+      </c>
+      <c r="B23" s="83" t="s">
+        <v>359</v>
+      </c>
+      <c r="C23" s="89" t="s">
+        <v>352</v>
+      </c>
+      <c r="D23" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="E23" s="92" t="s">
+        <v>357</v>
+      </c>
+      <c r="F23" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="68"/>
+      <c r="I23" s="96" t="s">
+        <v>437</v>
+      </c>
+      <c r="J23" s="96" t="s">
+        <v>436</v>
+      </c>
+      <c r="K23" s="56"/>
+      <c r="L23" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="M23" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="N23" s="98" t="s">
+        <v>442</v>
+      </c>
+      <c r="O23" s="87" t="s">
+        <v>351</v>
+      </c>
+      <c r="P23" s="70" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q23" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="R23" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="S23" s="57"/>
+      <c r="T23" s="58"/>
+      <c r="U23" s="58"/>
+      <c r="V23" s="58"/>
+      <c r="W23" s="58"/>
+      <c r="X23" s="58"/>
+      <c r="Y23" s="58"/>
+      <c r="Z23" s="58"/>
+      <c r="AA23" s="58"/>
+      <c r="AB23" s="58"/>
+      <c r="AC23" s="58"/>
+      <c r="AD23" s="58"/>
+      <c r="AE23" s="58"/>
+    </row>
+    <row r="24" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="61"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="56"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="70"/>
+      <c r="Q24" s="72"/>
+      <c r="R24" s="71"/>
+      <c r="S24" s="57"/>
+      <c r="T24" s="58"/>
+      <c r="U24" s="58"/>
+      <c r="V24" s="58"/>
+      <c r="W24" s="58"/>
+      <c r="X24" s="58"/>
+      <c r="Y24" s="58"/>
+      <c r="Z24" s="58"/>
+      <c r="AA24" s="58"/>
+      <c r="AB24" s="58"/>
+      <c r="AC24" s="58"/>
+      <c r="AD24" s="58"/>
+      <c r="AE24" s="58"/>
+    </row>
+    <row r="25" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="61"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="68"/>
+      <c r="I25" s="64"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="56"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="56"/>
+      <c r="N25" s="56"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="70"/>
+      <c r="Q25" s="72"/>
+      <c r="R25" s="71"/>
+      <c r="S25" s="57"/>
+      <c r="T25" s="58"/>
+      <c r="U25" s="58"/>
+      <c r="V25" s="58"/>
+      <c r="W25" s="58"/>
+      <c r="X25" s="58"/>
+      <c r="Y25" s="58"/>
+      <c r="Z25" s="58"/>
+      <c r="AA25" s="58"/>
+      <c r="AB25" s="58"/>
+      <c r="AC25" s="58"/>
+      <c r="AD25" s="58"/>
+      <c r="AE25" s="58"/>
+    </row>
+    <row r="26" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="65"/>
+      <c r="J26" s="52"/>
+      <c r="K26" s="56"/>
+      <c r="L26" s="56"/>
+      <c r="M26" s="56"/>
+      <c r="N26" s="56"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="70"/>
+      <c r="Q26" s="72"/>
+      <c r="R26" s="71"/>
+      <c r="S26" s="57"/>
+      <c r="T26" s="58"/>
+      <c r="U26" s="58"/>
+      <c r="V26" s="58"/>
+      <c r="W26" s="58"/>
+      <c r="X26" s="58"/>
+      <c r="Y26" s="58"/>
+      <c r="Z26" s="58"/>
+      <c r="AA26" s="58"/>
+      <c r="AB26" s="58"/>
+      <c r="AC26" s="58"/>
+      <c r="AD26" s="58"/>
+      <c r="AE26" s="58"/>
+    </row>
+    <row r="27" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="64"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="56"/>
+      <c r="L27" s="56"/>
+      <c r="M27" s="56"/>
+      <c r="N27" s="56"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="70"/>
+      <c r="Q27" s="72"/>
+      <c r="R27" s="71"/>
+      <c r="S27" s="57"/>
+      <c r="T27" s="58"/>
+      <c r="U27" s="58"/>
+      <c r="V27" s="58"/>
+      <c r="W27" s="58"/>
+      <c r="X27" s="58"/>
+      <c r="Y27" s="58"/>
+      <c r="Z27" s="58"/>
+      <c r="AA27" s="58"/>
+      <c r="AB27" s="58"/>
+      <c r="AC27" s="58"/>
+      <c r="AD27" s="58"/>
+      <c r="AE27" s="58"/>
+    </row>
+    <row r="28" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="69"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="52"/>
+      <c r="K28" s="56"/>
+      <c r="L28" s="56"/>
+      <c r="M28" s="56"/>
+      <c r="N28" s="56"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="70"/>
+      <c r="Q28" s="72"/>
+      <c r="R28" s="71"/>
+      <c r="S28" s="57"/>
+      <c r="T28" s="58"/>
+      <c r="U28" s="58"/>
+      <c r="V28" s="58"/>
+      <c r="W28" s="58"/>
+      <c r="X28" s="58"/>
+      <c r="Y28" s="58"/>
+      <c r="Z28" s="58"/>
+      <c r="AA28" s="58"/>
+      <c r="AB28" s="58"/>
+      <c r="AC28" s="58"/>
+      <c r="AD28" s="58"/>
+      <c r="AE28" s="58"/>
+    </row>
+    <row r="29" spans="1:31" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="68"/>
+      <c r="I29" s="64"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="56"/>
+      <c r="L29" s="56"/>
+      <c r="M29" s="56"/>
+      <c r="N29" s="56"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="70"/>
+      <c r="Q29" s="72"/>
+      <c r="R29" s="71"/>
+      <c r="S29" s="57"/>
+      <c r="T29" s="58"/>
+      <c r="U29" s="58"/>
+      <c r="V29" s="58"/>
+      <c r="W29" s="58"/>
+      <c r="X29" s="58"/>
+      <c r="Y29" s="58"/>
+      <c r="Z29" s="58"/>
+      <c r="AA29" s="58"/>
+      <c r="AB29" s="58"/>
+      <c r="AC29" s="58"/>
+      <c r="AD29" s="58"/>
+      <c r="AE29" s="58"/>
     </row>
     <row r="30" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E30" s="59"/>
@@ -5747,43 +6000,57 @@
     <row r="221" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E221" s="59"/>
       <c r="I221" s="59"/>
-      <c r="J221" s="59"/>
+      <c r="J221" s="60"/>
+      <c r="O221" s="60"/>
+      <c r="R221" s="60"/>
       <c r="S221" s="59"/>
     </row>
     <row r="222" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E222" s="59"/>
       <c r="I222" s="59"/>
-      <c r="J222" s="59"/>
+      <c r="J222" s="60"/>
+      <c r="O222" s="60"/>
+      <c r="R222" s="60"/>
       <c r="S222" s="59"/>
     </row>
     <row r="223" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E223" s="59"/>
       <c r="I223" s="59"/>
-      <c r="J223" s="59"/>
+      <c r="J223" s="60"/>
+      <c r="O223" s="60"/>
+      <c r="R223" s="60"/>
       <c r="S223" s="59"/>
     </row>
     <row r="224" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E224" s="59"/>
       <c r="I224" s="59"/>
-      <c r="J224" s="59"/>
+      <c r="J224" s="60"/>
+      <c r="O224" s="60"/>
+      <c r="R224" s="60"/>
       <c r="S224" s="59"/>
     </row>
     <row r="225" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E225" s="59"/>
       <c r="I225" s="59"/>
-      <c r="J225" s="59"/>
+      <c r="J225" s="60"/>
+      <c r="O225" s="60"/>
+      <c r="R225" s="60"/>
       <c r="S225" s="59"/>
     </row>
     <row r="226" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E226" s="59"/>
       <c r="I226" s="59"/>
-      <c r="J226" s="59"/>
+      <c r="J226" s="60"/>
+      <c r="O226" s="60"/>
+      <c r="R226" s="60"/>
       <c r="S226" s="59"/>
     </row>
     <row r="227" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E227" s="59"/>
       <c r="I227" s="59"/>
-      <c r="J227" s="59"/>
+      <c r="J227" s="60"/>
+      <c r="O227" s="60"/>
+      <c r="R227" s="60"/>
       <c r="S227" s="59"/>
     </row>
     <row r="228" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10424,82 +10691,78 @@
       <c r="J1000" s="59"/>
       <c r="S1000" s="59"/>
     </row>
+    <row r="1001" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1001" s="59"/>
+      <c r="I1001" s="59"/>
+      <c r="J1001" s="59"/>
+      <c r="S1001" s="59"/>
+    </row>
+    <row r="1002" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1002" s="59"/>
+      <c r="I1002" s="59"/>
+      <c r="J1002" s="59"/>
+      <c r="S1002" s="59"/>
+    </row>
+    <row r="1003" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1003" s="59"/>
+      <c r="I1003" s="59"/>
+      <c r="J1003" s="59"/>
+      <c r="S1003" s="59"/>
+    </row>
+    <row r="1004" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1004" s="59"/>
+      <c r="I1004" s="59"/>
+      <c r="J1004" s="59"/>
+      <c r="S1004" s="59"/>
+    </row>
+    <row r="1005" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1005" s="59"/>
+      <c r="I1005" s="59"/>
+      <c r="J1005" s="59"/>
+      <c r="S1005" s="59"/>
+    </row>
+    <row r="1006" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1006" s="59"/>
+      <c r="I1006" s="59"/>
+      <c r="J1006" s="59"/>
+      <c r="S1006" s="59"/>
+    </row>
+    <row r="1007" spans="5:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1007" s="59"/>
+      <c r="I1007" s="59"/>
+      <c r="J1007" s="59"/>
+      <c r="S1007" s="59"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="22" type="noConversion"/>
-  <conditionalFormatting sqref="Q19:Q22 Q2:Q11">
-    <cfRule type="containsText" dxfId="48" priority="15" operator="containsText" text="New">
+  <conditionalFormatting sqref="Q2:Q29">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="New">
       <formula>NOT(ISERROR(SEARCH("New",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="47" priority="16" operator="containsText" text="New">
+    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="New">
       <formula>NOT(ISERROR(SEARCH("New",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="17" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="18" operator="containsText" text="Fix">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Fix">
       <formula>NOT(ISERROR(SEARCH("Fix",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="19" operator="containsText" text="Reopen">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="Reopen">
       <formula>NOT(ISERROR(SEARCH("Reopen",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="20" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",Q2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="21" operator="containsText" text="Reopen">
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="Reopen">
       <formula>NOT(ISERROR(SEARCH("Reopen",Q2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q12">
-    <cfRule type="containsText" dxfId="41" priority="8" operator="containsText" text="New">
-      <formula>NOT(ISERROR(SEARCH("New",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="9" operator="containsText" text="New">
-      <formula>NOT(ISERROR(SEARCH("New",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="10" operator="containsText" text="Closed">
-      <formula>NOT(ISERROR(SEARCH("Closed",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="11" operator="containsText" text="Fix">
-      <formula>NOT(ISERROR(SEARCH("Fix",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="12" operator="containsText" text="Reopen">
-      <formula>NOT(ISERROR(SEARCH("Reopen",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="36" priority="13" operator="containsText" text="Open">
-      <formula>NOT(ISERROR(SEARCH("Open",Q12)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="35" priority="14" operator="containsText" text="Reopen">
-      <formula>NOT(ISERROR(SEARCH("Reopen",Q12)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q13:Q18">
-    <cfRule type="containsText" dxfId="34" priority="1" operator="containsText" text="New">
-      <formula>NOT(ISERROR(SEARCH("New",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="2" operator="containsText" text="New">
-      <formula>NOT(ISERROR(SEARCH("New",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="3" operator="containsText" text="Closed">
-      <formula>NOT(ISERROR(SEARCH("Closed",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="4" operator="containsText" text="Fix">
-      <formula>NOT(ISERROR(SEARCH("Fix",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="5" operator="containsText" text="Reopen">
-      <formula>NOT(ISERROR(SEARCH("Reopen",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="6" operator="containsText" text="Open">
-      <formula>NOT(ISERROR(SEARCH("Open",Q13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="7" operator="containsText" text="Reopen">
-      <formula>NOT(ISERROR(SEARCH("Reopen",Q13)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F22">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F29" xr:uid="{872A2AB6-2ADB-4D3A-9A56-79D755130126}">
       <formula1>"valid,invalid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q22">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q29" xr:uid="{7A9CF52A-021F-4101-8226-913AE7D0D2C0}">
       <formula1>"New, Open, Fix, Reopen, Closed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10509,7 +10772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -16033,20 +16296,20 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q2:Q979">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q2:Q979" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"not executed,blocked,failed,passed"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E5" r:id="rId4"/>
-    <hyperlink ref="E6" r:id="rId5"/>
-    <hyperlink ref="E7" r:id="rId6"/>
-    <hyperlink ref="E8" r:id="rId7"/>
-    <hyperlink ref="E9" r:id="rId8"/>
-    <hyperlink ref="E36" r:id="rId9"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="E36" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>